<commit_message>
Fix mapping et DroitDecision 782250e09855411da56baa807b9db2ebfd4978d1
</commit_message>
<xml_diff>
--- a/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-decision.xlsx
+++ b/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/StructureDefinition-tddui-decision.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5413" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5735" uniqueCount="388">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-12T15:13:13+00:00</t>
+    <t>2026-06-15T13:25:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -680,6 +680,30 @@
 </t>
   </si>
   <si>
+    <t>Extension.extension:decision.extension:droitPrestation.extension:motifFinPAG</t>
+  </si>
+  <si>
+    <t>motifFinPAG</t>
+  </si>
+  <si>
+    <t>Motif de fin du PAG</t>
+  </si>
+  <si>
+    <t>Extension.extension:decision.extension:droitPrestation.extension:motifFinPAG.id</t>
+  </si>
+  <si>
+    <t>Extension.extension:decision.extension:droitPrestation.extension:motifFinPAG.extension</t>
+  </si>
+  <si>
+    <t>Extension.extension:decision.extension:droitPrestation.extension:motifFinPAG.url</t>
+  </si>
+  <si>
+    <t>Extension.extension:decision.extension:droitPrestation.extension:motifFinPAG.value[x]</t>
+  </si>
+  <si>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-j403-motif-fin-pag-ms</t>
+  </si>
+  <si>
     <t>Extension.extension:decision.extension:droitPrestation.extension:creton</t>
   </si>
   <si>
@@ -726,6 +750,30 @@
 </t>
   </si>
   <si>
+    <t>Extension.extension:decision.extension:droitPrestation.extension:typeCompensation</t>
+  </si>
+  <si>
+    <t>typeCompensation</t>
+  </si>
+  <si>
+    <t>Type de compensation</t>
+  </si>
+  <si>
+    <t>Extension.extension:decision.extension:droitPrestation.extension:typeCompensation.id</t>
+  </si>
+  <si>
+    <t>Extension.extension:decision.extension:droitPrestation.extension:typeCompensation.extension</t>
+  </si>
+  <si>
+    <t>Extension.extension:decision.extension:droitPrestation.extension:typeCompensation.url</t>
+  </si>
+  <si>
+    <t>Extension.extension:decision.extension:droitPrestation.extension:typeCompensation.value[x]</t>
+  </si>
+  <si>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-j394-type-demande-compensation-ms</t>
+  </si>
+  <si>
     <t>Extension.extension:decision.extension:droitPrestation.extension:commentaire</t>
   </si>
   <si>
@@ -754,9 +802,6 @@
   </si>
   <si>
     <t>Extension.extension:decision.extension:droitPrestation.extension:detailPrestation.extension</t>
-  </si>
-  <si>
-    <t>2</t>
   </si>
   <si>
     <t>Extension.extension:decision.extension:droitPrestation.extension:detailPrestation.extension:temporaliteAccueil</t>
@@ -892,7 +937,7 @@
     <t>frequence</t>
   </si>
   <si>
-    <t>Fréquence</t>
+    <t>Fréquence de versement</t>
   </si>
   <si>
     <t>Extension.extension:decision.extension:droitPrestation.extension:detailPrestation.extension:frequence.id</t>
@@ -1458,7 +1503,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK166"/>
+  <dimension ref="A1:AK176"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="137.41796875" customWidth="true" bestFit="true"/>
@@ -9205,7 +9250,7 @@
         <v>76</v>
       </c>
       <c r="K75" t="s" s="2">
-        <v>217</v>
+        <v>119</v>
       </c>
       <c r="L75" t="s" s="2">
         <v>120</v>
@@ -9238,13 +9283,11 @@
         <v>76</v>
       </c>
       <c r="X75" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y75" t="s" s="2">
-        <v>76</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="Y75" s="2"/>
       <c r="Z75" t="s" s="2">
-        <v>76</v>
+        <v>225</v>
       </c>
       <c r="AA75" t="s" s="2">
         <v>76</v>
@@ -9282,13 +9325,13 @@
     </row>
     <row r="76">
       <c r="A76" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B76" t="s" s="2">
         <v>108</v>
       </c>
       <c r="C76" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D76" t="s" s="2">
         <v>76</v>
@@ -9313,7 +9356,7 @@
         <v>90</v>
       </c>
       <c r="L76" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="M76" t="s" s="2">
         <v>91</v>
@@ -9387,7 +9430,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B77" t="s" s="2">
         <v>172</v>
@@ -9490,7 +9533,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B78" t="s" s="2">
         <v>174</v>
@@ -9593,7 +9636,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B79" t="s" s="2">
         <v>176</v>
@@ -9636,7 +9679,7 @@
       </c>
       <c r="Q79" s="2"/>
       <c r="R79" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="S79" t="s" s="2">
         <v>76</v>
@@ -9698,7 +9741,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B80" t="s" s="2">
         <v>178</v>
@@ -9724,7 +9767,7 @@
         <v>76</v>
       </c>
       <c r="K80" t="s" s="2">
-        <v>232</v>
+        <v>217</v>
       </c>
       <c r="L80" t="s" s="2">
         <v>120</v>
@@ -9807,7 +9850,7 @@
         <v>108</v>
       </c>
       <c r="C81" t="s" s="2">
-        <v>157</v>
+        <v>234</v>
       </c>
       <c r="D81" t="s" s="2">
         <v>76</v>
@@ -9832,7 +9875,7 @@
         <v>90</v>
       </c>
       <c r="L81" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="M81" t="s" s="2">
         <v>91</v>
@@ -9906,7 +9949,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B82" t="s" s="2">
         <v>172</v>
@@ -10009,7 +10052,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B83" t="s" s="2">
         <v>174</v>
@@ -10112,7 +10155,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B84" t="s" s="2">
         <v>176</v>
@@ -10155,7 +10198,7 @@
       </c>
       <c r="Q84" s="2"/>
       <c r="R84" t="s" s="2">
-        <v>157</v>
+        <v>234</v>
       </c>
       <c r="S84" t="s" s="2">
         <v>76</v>
@@ -10217,7 +10260,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B85" t="s" s="2">
         <v>178</v>
@@ -10243,7 +10286,7 @@
         <v>76</v>
       </c>
       <c r="K85" t="s" s="2">
-        <v>84</v>
+        <v>240</v>
       </c>
       <c r="L85" t="s" s="2">
         <v>120</v>
@@ -10320,20 +10363,20 @@
     </row>
     <row r="86">
       <c r="A86" t="s" s="2">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B86" t="s" s="2">
         <v>108</v>
       </c>
       <c r="C86" t="s" s="2">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D86" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E86" s="2"/>
       <c r="F86" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G86" t="s" s="2">
         <v>83</v>
@@ -10351,7 +10394,7 @@
         <v>90</v>
       </c>
       <c r="L86" t="s" s="2">
-        <v>30</v>
+        <v>243</v>
       </c>
       <c r="M86" t="s" s="2">
         <v>91</v>
@@ -10425,7 +10468,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s" s="2">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B87" t="s" s="2">
         <v>172</v>
@@ -10528,7 +10571,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B88" t="s" s="2">
         <v>174</v>
@@ -10539,10 +10582,10 @@
       </c>
       <c r="E88" s="2"/>
       <c r="F88" t="s" s="2">
-        <v>243</v>
+        <v>77</v>
       </c>
       <c r="G88" t="s" s="2">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H88" t="s" s="2">
         <v>76</v>
@@ -10631,20 +10674,18 @@
     </row>
     <row r="89">
       <c r="A89" t="s" s="2">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="C89" t="s" s="2">
-        <v>245</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E89" s="2"/>
       <c r="F89" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G89" t="s" s="2">
         <v>83</v>
@@ -10659,22 +10700,24 @@
         <v>76</v>
       </c>
       <c r="K89" t="s" s="2">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="L89" t="s" s="2">
-        <v>246</v>
+        <v>112</v>
       </c>
       <c r="M89" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="N89" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N89" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O89" s="2"/>
       <c r="P89" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q89" s="2"/>
       <c r="R89" t="s" s="2">
-        <v>76</v>
+        <v>242</v>
       </c>
       <c r="S89" t="s" s="2">
         <v>76</v>
@@ -10716,22 +10759,22 @@
         <v>76</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="AG89" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="AH89" t="s" s="2">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="AI89" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ89" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AK89" t="s" s="2">
-        <v>76</v>
+        <v>116</v>
       </c>
     </row>
     <row r="90">
@@ -10739,7 +10782,7 @@
         <v>247</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>248</v>
+        <v>178</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -10762,13 +10805,13 @@
         <v>76</v>
       </c>
       <c r="K90" t="s" s="2">
-        <v>84</v>
+        <v>119</v>
       </c>
       <c r="L90" t="s" s="2">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="M90" t="s" s="2">
-        <v>86</v>
+        <v>121</v>
       </c>
       <c r="N90" s="2"/>
       <c r="O90" s="2"/>
@@ -10795,13 +10838,11 @@
         <v>76</v>
       </c>
       <c r="X90" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y90" t="s" s="2">
-        <v>76</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="Y90" s="2"/>
       <c r="Z90" t="s" s="2">
-        <v>76</v>
+        <v>248</v>
       </c>
       <c r="AA90" t="s" s="2">
         <v>76</v>
@@ -10819,7 +10860,7 @@
         <v>76</v>
       </c>
       <c r="AF90" t="s" s="2">
-        <v>87</v>
+        <v>124</v>
       </c>
       <c r="AG90" t="s" s="2">
         <v>77</v>
@@ -10831,10 +10872,10 @@
         <v>76</v>
       </c>
       <c r="AJ90" t="s" s="2">
-        <v>76</v>
+        <v>125</v>
       </c>
       <c r="AK90" t="s" s="2">
-        <v>88</v>
+        <v>116</v>
       </c>
     </row>
     <row r="91">
@@ -10842,9 +10883,11 @@
         <v>249</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>250</v>
-      </c>
-      <c r="C91" s="2"/>
+        <v>108</v>
+      </c>
+      <c r="C91" t="s" s="2">
+        <v>157</v>
+      </c>
       <c r="D91" t="s" s="2">
         <v>76</v>
       </c>
@@ -10853,7 +10896,7 @@
         <v>77</v>
       </c>
       <c r="G91" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H91" t="s" s="2">
         <v>76</v>
@@ -10868,7 +10911,7 @@
         <v>90</v>
       </c>
       <c r="L91" t="s" s="2">
-        <v>30</v>
+        <v>250</v>
       </c>
       <c r="M91" t="s" s="2">
         <v>91</v>
@@ -10910,16 +10953,16 @@
         <v>76</v>
       </c>
       <c r="AB91" t="s" s="2">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="AC91" t="s" s="2">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="AD91" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE91" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AF91" t="s" s="2">
         <v>95</v>
@@ -10945,7 +10988,7 @@
         <v>251</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>252</v>
+        <v>172</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -10953,7 +10996,7 @@
       </c>
       <c r="E92" s="2"/>
       <c r="F92" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G92" t="s" s="2">
         <v>83</v>
@@ -10968,24 +11011,22 @@
         <v>76</v>
       </c>
       <c r="K92" t="s" s="2">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="L92" t="s" s="2">
-        <v>112</v>
+        <v>85</v>
       </c>
       <c r="M92" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N92" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="N92" s="2"/>
       <c r="O92" s="2"/>
       <c r="P92" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q92" s="2"/>
       <c r="R92" t="s" s="2">
-        <v>245</v>
+        <v>76</v>
       </c>
       <c r="S92" t="s" s="2">
         <v>76</v>
@@ -11027,10 +11068,10 @@
         <v>76</v>
       </c>
       <c r="AF92" t="s" s="2">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="AG92" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AH92" t="s" s="2">
         <v>83</v>
@@ -11042,15 +11083,15 @@
         <v>76</v>
       </c>
       <c r="AK92" t="s" s="2">
-        <v>116</v>
+        <v>88</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s" s="2">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>254</v>
+        <v>174</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -11061,7 +11102,7 @@
         <v>77</v>
       </c>
       <c r="G93" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="H93" t="s" s="2">
         <v>76</v>
@@ -11073,13 +11114,13 @@
         <v>76</v>
       </c>
       <c r="K93" t="s" s="2">
-        <v>119</v>
+        <v>90</v>
       </c>
       <c r="L93" t="s" s="2">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="M93" t="s" s="2">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="N93" s="2"/>
       <c r="O93" s="2"/>
@@ -11106,62 +11147,62 @@
         <v>76</v>
       </c>
       <c r="X93" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="Y93" s="2"/>
+        <v>76</v>
+      </c>
+      <c r="Y93" t="s" s="2">
+        <v>76</v>
+      </c>
       <c r="Z93" t="s" s="2">
-        <v>255</v>
+        <v>76</v>
       </c>
       <c r="AA93" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AB93" t="s" s="2">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="AC93" t="s" s="2">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="AD93" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE93" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AF93" t="s" s="2">
-        <v>124</v>
+        <v>95</v>
       </c>
       <c r="AG93" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH93" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="AI93" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ93" t="s" s="2">
-        <v>125</v>
+        <v>81</v>
       </c>
       <c r="AK93" t="s" s="2">
-        <v>116</v>
+        <v>76</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s" s="2">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="C94" t="s" s="2">
-        <v>257</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E94" s="2"/>
       <c r="F94" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G94" t="s" s="2">
         <v>83</v>
@@ -11176,22 +11217,24 @@
         <v>76</v>
       </c>
       <c r="K94" t="s" s="2">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>258</v>
+        <v>112</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="N94" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N94" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O94" s="2"/>
       <c r="P94" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q94" s="2"/>
       <c r="R94" t="s" s="2">
-        <v>76</v>
+        <v>157</v>
       </c>
       <c r="S94" t="s" s="2">
         <v>76</v>
@@ -11233,30 +11276,30 @@
         <v>76</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="AG94" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="AH94" t="s" s="2">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="AI94" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ94" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AK94" t="s" s="2">
-        <v>76</v>
+        <v>116</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s" s="2">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>248</v>
+        <v>178</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -11282,10 +11325,10 @@
         <v>84</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>86</v>
+        <v>121</v>
       </c>
       <c r="N95" s="2"/>
       <c r="O95" s="2"/>
@@ -11336,7 +11379,7 @@
         <v>76</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>87</v>
+        <v>124</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>77</v>
@@ -11348,29 +11391,31 @@
         <v>76</v>
       </c>
       <c r="AJ95" t="s" s="2">
-        <v>76</v>
+        <v>125</v>
       </c>
       <c r="AK95" t="s" s="2">
-        <v>88</v>
+        <v>116</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>250</v>
-      </c>
-      <c r="C96" s="2"/>
+        <v>108</v>
+      </c>
+      <c r="C96" t="s" s="2">
+        <v>256</v>
+      </c>
       <c r="D96" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E96" s="2"/>
       <c r="F96" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G96" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H96" t="s" s="2">
         <v>76</v>
@@ -11427,16 +11472,16 @@
         <v>76</v>
       </c>
       <c r="AB96" t="s" s="2">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="AC96" t="s" s="2">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="AD96" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE96" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AF96" t="s" s="2">
         <v>95</v>
@@ -11459,10 +11504,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s" s="2">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>252</v>
+        <v>172</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -11470,7 +11515,7 @@
       </c>
       <c r="E97" s="2"/>
       <c r="F97" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G97" t="s" s="2">
         <v>83</v>
@@ -11485,24 +11530,22 @@
         <v>76</v>
       </c>
       <c r="K97" t="s" s="2">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="L97" t="s" s="2">
-        <v>112</v>
+        <v>85</v>
       </c>
       <c r="M97" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N97" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="N97" s="2"/>
       <c r="O97" s="2"/>
       <c r="P97" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q97" s="2"/>
       <c r="R97" t="s" s="2">
-        <v>257</v>
+        <v>76</v>
       </c>
       <c r="S97" t="s" s="2">
         <v>76</v>
@@ -11544,10 +11587,10 @@
         <v>76</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="AG97" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AH97" t="s" s="2">
         <v>83</v>
@@ -11559,15 +11602,15 @@
         <v>76</v>
       </c>
       <c r="AK97" t="s" s="2">
-        <v>116</v>
+        <v>88</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>254</v>
+        <v>174</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -11575,10 +11618,10 @@
       </c>
       <c r="E98" s="2"/>
       <c r="F98" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G98" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="H98" t="s" s="2">
         <v>76</v>
@@ -11590,13 +11633,13 @@
         <v>76</v>
       </c>
       <c r="K98" t="s" s="2">
-        <v>119</v>
+        <v>90</v>
       </c>
       <c r="L98" t="s" s="2">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="M98" t="s" s="2">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="N98" s="2"/>
       <c r="O98" s="2"/>
@@ -11623,55 +11666,57 @@
         <v>76</v>
       </c>
       <c r="X98" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="Y98" s="2"/>
+        <v>76</v>
+      </c>
+      <c r="Y98" t="s" s="2">
+        <v>76</v>
+      </c>
       <c r="Z98" t="s" s="2">
-        <v>263</v>
+        <v>76</v>
       </c>
       <c r="AA98" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AB98" t="s" s="2">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="AC98" t="s" s="2">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="AD98" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE98" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>124</v>
+        <v>95</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH98" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="AI98" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ98" t="s" s="2">
-        <v>125</v>
+        <v>81</v>
       </c>
       <c r="AK98" t="s" s="2">
-        <v>116</v>
+        <v>76</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s" s="2">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="B99" t="s" s="2">
         <v>174</v>
       </c>
       <c r="C99" t="s" s="2">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="D99" t="s" s="2">
         <v>76</v>
@@ -11696,7 +11741,7 @@
         <v>90</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="M99" t="s" s="2">
         <v>91</v>
@@ -11770,10 +11815,10 @@
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -11873,10 +11918,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -11976,10 +12021,10 @@
     </row>
     <row r="102">
       <c r="A102" t="s" s="2">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -12019,7 +12064,7 @@
       </c>
       <c r="Q102" s="2"/>
       <c r="R102" t="s" s="2">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="S102" t="s" s="2">
         <v>76</v>
@@ -12081,10 +12126,10 @@
     </row>
     <row r="103">
       <c r="A103" t="s" s="2">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -12107,7 +12152,7 @@
         <v>76</v>
       </c>
       <c r="K103" t="s" s="2">
-        <v>217</v>
+        <v>119</v>
       </c>
       <c r="L103" t="s" s="2">
         <v>120</v>
@@ -12140,13 +12185,11 @@
         <v>76</v>
       </c>
       <c r="X103" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y103" t="s" s="2">
-        <v>76</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="Y103" s="2"/>
       <c r="Z103" t="s" s="2">
-        <v>76</v>
+        <v>270</v>
       </c>
       <c r="AA103" t="s" s="2">
         <v>76</v>
@@ -12292,7 +12335,7 @@
         <v>274</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -12395,7 +12438,7 @@
         <v>275</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -12498,7 +12541,7 @@
         <v>276</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -12603,7 +12646,7 @@
         <v>277</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -12626,7 +12669,7 @@
         <v>76</v>
       </c>
       <c r="K108" t="s" s="2">
-        <v>84</v>
+        <v>119</v>
       </c>
       <c r="L108" t="s" s="2">
         <v>120</v>
@@ -12659,13 +12702,11 @@
         <v>76</v>
       </c>
       <c r="X108" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y108" t="s" s="2">
-        <v>76</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="Y108" s="2"/>
       <c r="Z108" t="s" s="2">
-        <v>76</v>
+        <v>278</v>
       </c>
       <c r="AA108" t="s" s="2">
         <v>76</v>
@@ -12703,13 +12744,13 @@
     </row>
     <row r="109">
       <c r="A109" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B109" t="s" s="2">
         <v>174</v>
       </c>
       <c r="C109" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D109" t="s" s="2">
         <v>76</v>
@@ -12734,7 +12775,7 @@
         <v>90</v>
       </c>
       <c r="L109" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="M109" t="s" s="2">
         <v>91</v>
@@ -12808,10 +12849,10 @@
     </row>
     <row r="110">
       <c r="A110" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -12911,10 +12952,10 @@
     </row>
     <row r="111">
       <c r="A111" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
@@ -13014,10 +13055,10 @@
     </row>
     <row r="112">
       <c r="A112" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -13057,7 +13098,7 @@
       </c>
       <c r="Q112" s="2"/>
       <c r="R112" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="S112" t="s" s="2">
         <v>76</v>
@@ -13119,10 +13160,10 @@
     </row>
     <row r="113">
       <c r="A113" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -13145,7 +13186,7 @@
         <v>76</v>
       </c>
       <c r="K113" t="s" s="2">
-        <v>285</v>
+        <v>217</v>
       </c>
       <c r="L113" t="s" s="2">
         <v>120</v>
@@ -13330,7 +13371,7 @@
         <v>289</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
@@ -13433,7 +13474,7 @@
         <v>290</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -13536,7 +13577,7 @@
         <v>291</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -13641,7 +13682,7 @@
         <v>292</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" t="s" s="2">
@@ -13664,7 +13705,7 @@
         <v>76</v>
       </c>
       <c r="K118" t="s" s="2">
-        <v>232</v>
+        <v>84</v>
       </c>
       <c r="L118" t="s" s="2">
         <v>120</v>
@@ -13754,7 +13795,7 @@
       </c>
       <c r="E119" s="2"/>
       <c r="F119" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G119" t="s" s="2">
         <v>83</v>
@@ -13849,7 +13890,7 @@
         <v>296</v>
       </c>
       <c r="B120" t="s" s="2">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="C120" s="2"/>
       <c r="D120" t="s" s="2">
@@ -13952,7 +13993,7 @@
         <v>297</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
@@ -14055,7 +14096,7 @@
         <v>298</v>
       </c>
       <c r="B122" t="s" s="2">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" t="s" s="2">
@@ -14160,7 +14201,7 @@
         <v>299</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
@@ -14183,7 +14224,7 @@
         <v>76</v>
       </c>
       <c r="K123" t="s" s="2">
-        <v>119</v>
+        <v>300</v>
       </c>
       <c r="L123" t="s" s="2">
         <v>120</v>
@@ -14216,11 +14257,13 @@
         <v>76</v>
       </c>
       <c r="X123" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="Y123" s="2"/>
+        <v>76</v>
+      </c>
+      <c r="Y123" t="s" s="2">
+        <v>76</v>
+      </c>
       <c r="Z123" t="s" s="2">
-        <v>300</v>
+        <v>76</v>
       </c>
       <c r="AA123" t="s" s="2">
         <v>76</v>
@@ -14271,10 +14314,10 @@
       </c>
       <c r="E124" s="2"/>
       <c r="F124" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G124" t="s" s="2">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="H124" t="s" s="2">
         <v>76</v>
@@ -14366,7 +14409,7 @@
         <v>304</v>
       </c>
       <c r="B125" t="s" s="2">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" t="s" s="2">
@@ -14469,7 +14512,7 @@
         <v>305</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -14572,7 +14615,7 @@
         <v>306</v>
       </c>
       <c r="B127" t="s" s="2">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
@@ -14677,7 +14720,7 @@
         <v>307</v>
       </c>
       <c r="B128" t="s" s="2">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="C128" s="2"/>
       <c r="D128" t="s" s="2">
@@ -14700,7 +14743,7 @@
         <v>76</v>
       </c>
       <c r="K128" t="s" s="2">
-        <v>308</v>
+        <v>240</v>
       </c>
       <c r="L128" t="s" s="2">
         <v>120</v>
@@ -14777,23 +14820,23 @@
     </row>
     <row r="129">
       <c r="A129" t="s" s="2">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B129" t="s" s="2">
         <v>174</v>
       </c>
       <c r="C129" t="s" s="2">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D129" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E129" s="2"/>
       <c r="F129" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G129" t="s" s="2">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="H129" t="s" s="2">
         <v>76</v>
@@ -14808,7 +14851,7 @@
         <v>90</v>
       </c>
       <c r="L129" t="s" s="2">
-        <v>30</v>
+        <v>310</v>
       </c>
       <c r="M129" t="s" s="2">
         <v>91</v>
@@ -14885,7 +14928,7 @@
         <v>311</v>
       </c>
       <c r="B130" t="s" s="2">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="C130" s="2"/>
       <c r="D130" t="s" s="2">
@@ -14988,18 +15031,18 @@
         <v>312</v>
       </c>
       <c r="B131" t="s" s="2">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="C131" s="2"/>
       <c r="D131" t="s" s="2">
-        <v>313</v>
+        <v>76</v>
       </c>
       <c r="E131" s="2"/>
       <c r="F131" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G131" t="s" s="2">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H131" t="s" s="2">
         <v>76</v>
@@ -15014,14 +15057,12 @@
         <v>90</v>
       </c>
       <c r="L131" t="s" s="2">
-        <v>314</v>
+        <v>30</v>
       </c>
       <c r="M131" t="s" s="2">
-        <v>315</v>
-      </c>
-      <c r="N131" t="s" s="2">
-        <v>316</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="N131" s="2"/>
       <c r="O131" s="2"/>
       <c r="P131" t="s" s="2">
         <v>76</v>
@@ -15085,25 +15126,23 @@
         <v>81</v>
       </c>
       <c r="AK131" t="s" s="2">
-        <v>88</v>
+        <v>76</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="s" s="2">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="B132" t="s" s="2">
-        <v>250</v>
-      </c>
-      <c r="C132" t="s" s="2">
-        <v>318</v>
-      </c>
+        <v>267</v>
+      </c>
+      <c r="C132" s="2"/>
       <c r="D132" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E132" s="2"/>
       <c r="F132" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G132" t="s" s="2">
         <v>83</v>
@@ -15118,22 +15157,24 @@
         <v>76</v>
       </c>
       <c r="K132" t="s" s="2">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="L132" t="s" s="2">
-        <v>319</v>
+        <v>112</v>
       </c>
       <c r="M132" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="N132" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N132" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O132" s="2"/>
       <c r="P132" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q132" s="2"/>
       <c r="R132" t="s" s="2">
-        <v>76</v>
+        <v>309</v>
       </c>
       <c r="S132" t="s" s="2">
         <v>76</v>
@@ -15175,30 +15216,30 @@
         <v>76</v>
       </c>
       <c r="AF132" t="s" s="2">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="AG132" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="AH132" t="s" s="2">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="AI132" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ132" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AK132" t="s" s="2">
-        <v>76</v>
+        <v>116</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="s" s="2">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="B133" t="s" s="2">
-        <v>321</v>
+        <v>269</v>
       </c>
       <c r="C133" s="2"/>
       <c r="D133" t="s" s="2">
@@ -15221,13 +15262,13 @@
         <v>76</v>
       </c>
       <c r="K133" t="s" s="2">
-        <v>84</v>
+        <v>119</v>
       </c>
       <c r="L133" t="s" s="2">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="M133" t="s" s="2">
-        <v>86</v>
+        <v>121</v>
       </c>
       <c r="N133" s="2"/>
       <c r="O133" s="2"/>
@@ -15254,13 +15295,11 @@
         <v>76</v>
       </c>
       <c r="X133" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y133" t="s" s="2">
-        <v>76</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="Y133" s="2"/>
       <c r="Z133" t="s" s="2">
-        <v>76</v>
+        <v>315</v>
       </c>
       <c r="AA133" t="s" s="2">
         <v>76</v>
@@ -15278,7 +15317,7 @@
         <v>76</v>
       </c>
       <c r="AF133" t="s" s="2">
-        <v>87</v>
+        <v>124</v>
       </c>
       <c r="AG133" t="s" s="2">
         <v>77</v>
@@ -15290,20 +15329,22 @@
         <v>76</v>
       </c>
       <c r="AJ133" t="s" s="2">
-        <v>76</v>
+        <v>125</v>
       </c>
       <c r="AK133" t="s" s="2">
-        <v>88</v>
+        <v>116</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="s" s="2">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="B134" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="C134" s="2"/>
+        <v>174</v>
+      </c>
+      <c r="C134" t="s" s="2">
+        <v>317</v>
+      </c>
       <c r="D134" t="s" s="2">
         <v>76</v>
       </c>
@@ -15312,7 +15353,7 @@
         <v>77</v>
       </c>
       <c r="G134" t="s" s="2">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H134" t="s" s="2">
         <v>76</v>
@@ -15327,7 +15368,7 @@
         <v>90</v>
       </c>
       <c r="L134" t="s" s="2">
-        <v>30</v>
+        <v>318</v>
       </c>
       <c r="M134" t="s" s="2">
         <v>91</v>
@@ -15369,16 +15410,16 @@
         <v>76</v>
       </c>
       <c r="AB134" t="s" s="2">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="AC134" t="s" s="2">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="AD134" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE134" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AF134" t="s" s="2">
         <v>95</v>
@@ -15401,10 +15442,10 @@
     </row>
     <row r="135">
       <c r="A135" t="s" s="2">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B135" t="s" s="2">
-        <v>325</v>
+        <v>263</v>
       </c>
       <c r="C135" s="2"/>
       <c r="D135" t="s" s="2">
@@ -15412,7 +15453,7 @@
       </c>
       <c r="E135" s="2"/>
       <c r="F135" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G135" t="s" s="2">
         <v>83</v>
@@ -15427,24 +15468,22 @@
         <v>76</v>
       </c>
       <c r="K135" t="s" s="2">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="L135" t="s" s="2">
-        <v>112</v>
+        <v>85</v>
       </c>
       <c r="M135" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N135" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="N135" s="2"/>
       <c r="O135" s="2"/>
       <c r="P135" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q135" s="2"/>
       <c r="R135" t="s" s="2">
-        <v>318</v>
+        <v>76</v>
       </c>
       <c r="S135" t="s" s="2">
         <v>76</v>
@@ -15486,10 +15525,10 @@
         <v>76</v>
       </c>
       <c r="AF135" t="s" s="2">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="AG135" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AH135" t="s" s="2">
         <v>83</v>
@@ -15501,15 +15540,15 @@
         <v>76</v>
       </c>
       <c r="AK135" t="s" s="2">
-        <v>116</v>
+        <v>88</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="s" s="2">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="B136" t="s" s="2">
-        <v>327</v>
+        <v>265</v>
       </c>
       <c r="C136" s="2"/>
       <c r="D136" t="s" s="2">
@@ -15520,7 +15559,7 @@
         <v>77</v>
       </c>
       <c r="G136" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="H136" t="s" s="2">
         <v>76</v>
@@ -15532,13 +15571,13 @@
         <v>76</v>
       </c>
       <c r="K136" t="s" s="2">
-        <v>119</v>
+        <v>90</v>
       </c>
       <c r="L136" t="s" s="2">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="M136" t="s" s="2">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="N136" s="2"/>
       <c r="O136" s="2"/>
@@ -15565,62 +15604,62 @@
         <v>76</v>
       </c>
       <c r="X136" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="Y136" s="2"/>
+        <v>76</v>
+      </c>
+      <c r="Y136" t="s" s="2">
+        <v>76</v>
+      </c>
       <c r="Z136" t="s" s="2">
-        <v>328</v>
+        <v>76</v>
       </c>
       <c r="AA136" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AB136" t="s" s="2">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="AC136" t="s" s="2">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="AD136" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE136" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AF136" t="s" s="2">
-        <v>124</v>
+        <v>95</v>
       </c>
       <c r="AG136" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH136" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="AI136" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ136" t="s" s="2">
-        <v>125</v>
+        <v>81</v>
       </c>
       <c r="AK136" t="s" s="2">
-        <v>116</v>
+        <v>76</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="s" s="2">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="B137" t="s" s="2">
-        <v>250</v>
-      </c>
-      <c r="C137" t="s" s="2">
-        <v>330</v>
-      </c>
+        <v>267</v>
+      </c>
+      <c r="C137" s="2"/>
       <c r="D137" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E137" s="2"/>
       <c r="F137" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G137" t="s" s="2">
         <v>83</v>
@@ -15635,22 +15674,24 @@
         <v>76</v>
       </c>
       <c r="K137" t="s" s="2">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="L137" t="s" s="2">
-        <v>30</v>
+        <v>112</v>
       </c>
       <c r="M137" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="N137" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N137" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O137" s="2"/>
       <c r="P137" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q137" s="2"/>
       <c r="R137" t="s" s="2">
-        <v>76</v>
+        <v>317</v>
       </c>
       <c r="S137" t="s" s="2">
         <v>76</v>
@@ -15692,30 +15733,30 @@
         <v>76</v>
       </c>
       <c r="AF137" t="s" s="2">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="AG137" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="AH137" t="s" s="2">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="AI137" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ137" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AK137" t="s" s="2">
-        <v>76</v>
+        <v>116</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="s" s="2">
-        <v>331</v>
+        <v>322</v>
       </c>
       <c r="B138" t="s" s="2">
-        <v>321</v>
+        <v>269</v>
       </c>
       <c r="C138" s="2"/>
       <c r="D138" t="s" s="2">
@@ -15738,13 +15779,13 @@
         <v>76</v>
       </c>
       <c r="K138" t="s" s="2">
-        <v>84</v>
+        <v>323</v>
       </c>
       <c r="L138" t="s" s="2">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="M138" t="s" s="2">
-        <v>86</v>
+        <v>121</v>
       </c>
       <c r="N138" s="2"/>
       <c r="O138" s="2"/>
@@ -15795,7 +15836,7 @@
         <v>76</v>
       </c>
       <c r="AF138" t="s" s="2">
-        <v>87</v>
+        <v>124</v>
       </c>
       <c r="AG138" t="s" s="2">
         <v>77</v>
@@ -15807,22 +15848,24 @@
         <v>76</v>
       </c>
       <c r="AJ138" t="s" s="2">
-        <v>76</v>
+        <v>125</v>
       </c>
       <c r="AK138" t="s" s="2">
-        <v>88</v>
+        <v>116</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="s" s="2">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="B139" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="C139" s="2"/>
+        <v>174</v>
+      </c>
+      <c r="C139" t="s" s="2">
+        <v>325</v>
+      </c>
       <c r="D139" t="s" s="2">
-        <v>313</v>
+        <v>76</v>
       </c>
       <c r="E139" s="2"/>
       <c r="F139" t="s" s="2">
@@ -15844,14 +15887,12 @@
         <v>90</v>
       </c>
       <c r="L139" t="s" s="2">
-        <v>314</v>
+        <v>30</v>
       </c>
       <c r="M139" t="s" s="2">
-        <v>315</v>
-      </c>
-      <c r="N139" t="s" s="2">
-        <v>316</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="N139" s="2"/>
       <c r="O139" s="2"/>
       <c r="P139" t="s" s="2">
         <v>76</v>
@@ -15888,16 +15929,16 @@
         <v>76</v>
       </c>
       <c r="AB139" t="s" s="2">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="AC139" t="s" s="2">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="AD139" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE139" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AF139" t="s" s="2">
         <v>95</v>
@@ -15915,19 +15956,17 @@
         <v>81</v>
       </c>
       <c r="AK139" t="s" s="2">
-        <v>88</v>
+        <v>76</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="s" s="2">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="B140" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="C140" t="s" s="2">
-        <v>334</v>
-      </c>
+        <v>263</v>
+      </c>
+      <c r="C140" s="2"/>
       <c r="D140" t="s" s="2">
         <v>76</v>
       </c>
@@ -15948,13 +15987,13 @@
         <v>76</v>
       </c>
       <c r="K140" t="s" s="2">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="L140" t="s" s="2">
-        <v>335</v>
+        <v>85</v>
       </c>
       <c r="M140" t="s" s="2">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="N140" s="2"/>
       <c r="O140" s="2"/>
@@ -16005,41 +16044,41 @@
         <v>76</v>
       </c>
       <c r="AF140" t="s" s="2">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="AG140" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH140" t="s" s="2">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="AI140" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ140" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AK140" t="s" s="2">
-        <v>76</v>
+        <v>88</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="s" s="2">
-        <v>336</v>
+        <v>327</v>
       </c>
       <c r="B141" t="s" s="2">
-        <v>337</v>
+        <v>265</v>
       </c>
       <c r="C141" s="2"/>
       <c r="D141" t="s" s="2">
-        <v>76</v>
+        <v>328</v>
       </c>
       <c r="E141" s="2"/>
       <c r="F141" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G141" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="H141" t="s" s="2">
         <v>76</v>
@@ -16051,15 +16090,17 @@
         <v>76</v>
       </c>
       <c r="K141" t="s" s="2">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="L141" t="s" s="2">
-        <v>85</v>
+        <v>329</v>
       </c>
       <c r="M141" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="N141" s="2"/>
+        <v>330</v>
+      </c>
+      <c r="N141" t="s" s="2">
+        <v>331</v>
+      </c>
       <c r="O141" s="2"/>
       <c r="P141" t="s" s="2">
         <v>76</v>
@@ -16096,31 +16137,31 @@
         <v>76</v>
       </c>
       <c r="AB141" t="s" s="2">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="AC141" t="s" s="2">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="AD141" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE141" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AF141" t="s" s="2">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="AG141" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH141" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="AI141" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ141" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AK141" t="s" s="2">
         <v>88</v>
@@ -16128,12 +16169,14 @@
     </row>
     <row r="142">
       <c r="A142" t="s" s="2">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="B142" t="s" s="2">
-        <v>339</v>
-      </c>
-      <c r="C142" s="2"/>
+        <v>265</v>
+      </c>
+      <c r="C142" t="s" s="2">
+        <v>333</v>
+      </c>
       <c r="D142" t="s" s="2">
         <v>76</v>
       </c>
@@ -16142,7 +16185,7 @@
         <v>77</v>
       </c>
       <c r="G142" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H142" t="s" s="2">
         <v>76</v>
@@ -16157,7 +16200,7 @@
         <v>90</v>
       </c>
       <c r="L142" t="s" s="2">
-        <v>30</v>
+        <v>334</v>
       </c>
       <c r="M142" t="s" s="2">
         <v>91</v>
@@ -16199,16 +16242,16 @@
         <v>76</v>
       </c>
       <c r="AB142" t="s" s="2">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="AC142" t="s" s="2">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="AD142" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE142" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AF142" t="s" s="2">
         <v>95</v>
@@ -16231,10 +16274,10 @@
     </row>
     <row r="143">
       <c r="A143" t="s" s="2">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="B143" t="s" s="2">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C143" s="2"/>
       <c r="D143" t="s" s="2">
@@ -16242,7 +16285,7 @@
       </c>
       <c r="E143" s="2"/>
       <c r="F143" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G143" t="s" s="2">
         <v>83</v>
@@ -16257,24 +16300,22 @@
         <v>76</v>
       </c>
       <c r="K143" t="s" s="2">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="L143" t="s" s="2">
-        <v>112</v>
+        <v>85</v>
       </c>
       <c r="M143" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N143" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="N143" s="2"/>
       <c r="O143" s="2"/>
       <c r="P143" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q143" s="2"/>
       <c r="R143" t="s" s="2">
-        <v>334</v>
+        <v>76</v>
       </c>
       <c r="S143" t="s" s="2">
         <v>76</v>
@@ -16316,10 +16357,10 @@
         <v>76</v>
       </c>
       <c r="AF143" t="s" s="2">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="AG143" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AH143" t="s" s="2">
         <v>83</v>
@@ -16331,15 +16372,15 @@
         <v>76</v>
       </c>
       <c r="AK143" t="s" s="2">
-        <v>116</v>
+        <v>88</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="s" s="2">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="B144" t="s" s="2">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C144" s="2"/>
       <c r="D144" t="s" s="2">
@@ -16350,7 +16391,7 @@
         <v>77</v>
       </c>
       <c r="G144" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="H144" t="s" s="2">
         <v>76</v>
@@ -16362,13 +16403,13 @@
         <v>76</v>
       </c>
       <c r="K144" t="s" s="2">
-        <v>344</v>
+        <v>90</v>
       </c>
       <c r="L144" t="s" s="2">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="M144" t="s" s="2">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="N144" s="2"/>
       <c r="O144" s="2"/>
@@ -16407,52 +16448,50 @@
         <v>76</v>
       </c>
       <c r="AB144" t="s" s="2">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="AC144" t="s" s="2">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="AD144" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE144" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AF144" t="s" s="2">
-        <v>124</v>
+        <v>95</v>
       </c>
       <c r="AG144" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH144" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="AI144" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ144" t="s" s="2">
-        <v>125</v>
+        <v>81</v>
       </c>
       <c r="AK144" t="s" s="2">
-        <v>116</v>
+        <v>76</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="s" s="2">
-        <v>345</v>
+        <v>339</v>
       </c>
       <c r="B145" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="C145" t="s" s="2">
-        <v>346</v>
-      </c>
+        <v>340</v>
+      </c>
+      <c r="C145" s="2"/>
       <c r="D145" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E145" s="2"/>
       <c r="F145" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G145" t="s" s="2">
         <v>83</v>
@@ -16467,22 +16506,24 @@
         <v>76</v>
       </c>
       <c r="K145" t="s" s="2">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="L145" t="s" s="2">
-        <v>347</v>
+        <v>112</v>
       </c>
       <c r="M145" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="N145" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N145" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O145" s="2"/>
       <c r="P145" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q145" s="2"/>
       <c r="R145" t="s" s="2">
-        <v>76</v>
+        <v>333</v>
       </c>
       <c r="S145" t="s" s="2">
         <v>76</v>
@@ -16524,30 +16565,30 @@
         <v>76</v>
       </c>
       <c r="AF145" t="s" s="2">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="AG145" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="AH145" t="s" s="2">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="AI145" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ145" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AK145" t="s" s="2">
-        <v>76</v>
+        <v>116</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="s" s="2">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="B146" t="s" s="2">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="C146" s="2"/>
       <c r="D146" t="s" s="2">
@@ -16570,13 +16611,13 @@
         <v>76</v>
       </c>
       <c r="K146" t="s" s="2">
-        <v>84</v>
+        <v>119</v>
       </c>
       <c r="L146" t="s" s="2">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="M146" t="s" s="2">
-        <v>86</v>
+        <v>121</v>
       </c>
       <c r="N146" s="2"/>
       <c r="O146" s="2"/>
@@ -16603,13 +16644,11 @@
         <v>76</v>
       </c>
       <c r="X146" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y146" t="s" s="2">
-        <v>76</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="Y146" s="2"/>
       <c r="Z146" t="s" s="2">
-        <v>76</v>
+        <v>343</v>
       </c>
       <c r="AA146" t="s" s="2">
         <v>76</v>
@@ -16627,7 +16666,7 @@
         <v>76</v>
       </c>
       <c r="AF146" t="s" s="2">
-        <v>87</v>
+        <v>124</v>
       </c>
       <c r="AG146" t="s" s="2">
         <v>77</v>
@@ -16639,20 +16678,22 @@
         <v>76</v>
       </c>
       <c r="AJ146" t="s" s="2">
-        <v>76</v>
+        <v>125</v>
       </c>
       <c r="AK146" t="s" s="2">
-        <v>88</v>
+        <v>116</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="s" s="2">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="B147" t="s" s="2">
-        <v>339</v>
-      </c>
-      <c r="C147" s="2"/>
+        <v>265</v>
+      </c>
+      <c r="C147" t="s" s="2">
+        <v>345</v>
+      </c>
       <c r="D147" t="s" s="2">
         <v>76</v>
       </c>
@@ -16661,7 +16702,7 @@
         <v>77</v>
       </c>
       <c r="G147" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H147" t="s" s="2">
         <v>76</v>
@@ -16718,16 +16759,16 @@
         <v>76</v>
       </c>
       <c r="AB147" t="s" s="2">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="AC147" t="s" s="2">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="AD147" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE147" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AF147" t="s" s="2">
         <v>95</v>
@@ -16750,10 +16791,10 @@
     </row>
     <row r="148">
       <c r="A148" t="s" s="2">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="B148" t="s" s="2">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C148" s="2"/>
       <c r="D148" t="s" s="2">
@@ -16761,7 +16802,7 @@
       </c>
       <c r="E148" s="2"/>
       <c r="F148" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G148" t="s" s="2">
         <v>83</v>
@@ -16776,24 +16817,22 @@
         <v>76</v>
       </c>
       <c r="K148" t="s" s="2">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="L148" t="s" s="2">
-        <v>112</v>
+        <v>85</v>
       </c>
       <c r="M148" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N148" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="N148" s="2"/>
       <c r="O148" s="2"/>
       <c r="P148" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q148" s="2"/>
       <c r="R148" t="s" s="2">
-        <v>346</v>
+        <v>76</v>
       </c>
       <c r="S148" t="s" s="2">
         <v>76</v>
@@ -16835,10 +16874,10 @@
         <v>76</v>
       </c>
       <c r="AF148" t="s" s="2">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="AG148" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AH148" t="s" s="2">
         <v>83</v>
@@ -16850,26 +16889,26 @@
         <v>76</v>
       </c>
       <c r="AK148" t="s" s="2">
-        <v>116</v>
+        <v>88</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="s" s="2">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="B149" t="s" s="2">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C149" s="2"/>
       <c r="D149" t="s" s="2">
-        <v>76</v>
+        <v>328</v>
       </c>
       <c r="E149" s="2"/>
       <c r="F149" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G149" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="H149" t="s" s="2">
         <v>76</v>
@@ -16881,15 +16920,17 @@
         <v>76</v>
       </c>
       <c r="K149" t="s" s="2">
-        <v>232</v>
+        <v>90</v>
       </c>
       <c r="L149" t="s" s="2">
-        <v>120</v>
+        <v>329</v>
       </c>
       <c r="M149" t="s" s="2">
-        <v>121</v>
-      </c>
-      <c r="N149" s="2"/>
+        <v>330</v>
+      </c>
+      <c r="N149" t="s" s="2">
+        <v>331</v>
+      </c>
       <c r="O149" s="2"/>
       <c r="P149" t="s" s="2">
         <v>76</v>
@@ -16926,45 +16967,45 @@
         <v>76</v>
       </c>
       <c r="AB149" t="s" s="2">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="AC149" t="s" s="2">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="AD149" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE149" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AF149" t="s" s="2">
-        <v>124</v>
+        <v>95</v>
       </c>
       <c r="AG149" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH149" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="AI149" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ149" t="s" s="2">
-        <v>125</v>
+        <v>81</v>
       </c>
       <c r="AK149" t="s" s="2">
-        <v>116</v>
+        <v>88</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="s" s="2">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="B150" t="s" s="2">
-        <v>323</v>
+        <v>338</v>
       </c>
       <c r="C150" t="s" s="2">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="D150" t="s" s="2">
         <v>76</v>
@@ -16989,7 +17030,7 @@
         <v>90</v>
       </c>
       <c r="L150" t="s" s="2">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="M150" t="s" s="2">
         <v>91</v>
@@ -17063,10 +17104,10 @@
     </row>
     <row r="151">
       <c r="A151" t="s" s="2">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="B151" t="s" s="2">
-        <v>337</v>
+        <v>352</v>
       </c>
       <c r="C151" s="2"/>
       <c r="D151" t="s" s="2">
@@ -17166,10 +17207,10 @@
     </row>
     <row r="152">
       <c r="A152" t="s" s="2">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="B152" t="s" s="2">
-        <v>339</v>
+        <v>354</v>
       </c>
       <c r="C152" s="2"/>
       <c r="D152" t="s" s="2">
@@ -17269,10 +17310,10 @@
     </row>
     <row r="153">
       <c r="A153" t="s" s="2">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B153" t="s" s="2">
-        <v>341</v>
+        <v>356</v>
       </c>
       <c r="C153" s="2"/>
       <c r="D153" t="s" s="2">
@@ -17312,7 +17353,7 @@
       </c>
       <c r="Q153" s="2"/>
       <c r="R153" t="s" s="2">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="S153" t="s" s="2">
         <v>76</v>
@@ -17374,10 +17415,10 @@
     </row>
     <row r="154">
       <c r="A154" t="s" s="2">
+        <v>357</v>
+      </c>
+      <c r="B154" t="s" s="2">
         <v>358</v>
-      </c>
-      <c r="B154" t="s" s="2">
-        <v>343</v>
       </c>
       <c r="C154" s="2"/>
       <c r="D154" t="s" s="2">
@@ -17400,7 +17441,7 @@
         <v>76</v>
       </c>
       <c r="K154" t="s" s="2">
-        <v>119</v>
+        <v>359</v>
       </c>
       <c r="L154" t="s" s="2">
         <v>120</v>
@@ -17433,11 +17474,13 @@
         <v>76</v>
       </c>
       <c r="X154" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="Y154" s="2"/>
+        <v>76</v>
+      </c>
+      <c r="Y154" t="s" s="2">
+        <v>76</v>
+      </c>
       <c r="Z154" t="s" s="2">
-        <v>359</v>
+        <v>76</v>
       </c>
       <c r="AA154" t="s" s="2">
         <v>76</v>
@@ -17478,15 +17521,17 @@
         <v>360</v>
       </c>
       <c r="B155" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="C155" s="2"/>
+        <v>338</v>
+      </c>
+      <c r="C155" t="s" s="2">
+        <v>361</v>
+      </c>
       <c r="D155" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E155" s="2"/>
       <c r="F155" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G155" t="s" s="2">
         <v>83</v>
@@ -17501,24 +17546,22 @@
         <v>76</v>
       </c>
       <c r="K155" t="s" s="2">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="L155" t="s" s="2">
-        <v>112</v>
+        <v>362</v>
       </c>
       <c r="M155" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N155" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="N155" s="2"/>
       <c r="O155" s="2"/>
       <c r="P155" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q155" s="2"/>
       <c r="R155" t="s" s="2">
-        <v>330</v>
+        <v>76</v>
       </c>
       <c r="S155" t="s" s="2">
         <v>76</v>
@@ -17560,30 +17603,30 @@
         <v>76</v>
       </c>
       <c r="AF155" t="s" s="2">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="AG155" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AH155" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="AI155" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ155" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AK155" t="s" s="2">
-        <v>116</v>
+        <v>76</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="s" s="2">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B156" t="s" s="2">
-        <v>327</v>
+        <v>352</v>
       </c>
       <c r="C156" s="2"/>
       <c r="D156" t="s" s="2">
@@ -17594,7 +17637,7 @@
         <v>77</v>
       </c>
       <c r="G156" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H156" t="s" s="2">
         <v>76</v>
@@ -17606,13 +17649,13 @@
         <v>76</v>
       </c>
       <c r="K156" t="s" s="2">
-        <v>362</v>
+        <v>84</v>
       </c>
       <c r="L156" t="s" s="2">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="M156" t="s" s="2">
-        <v>121</v>
+        <v>86</v>
       </c>
       <c r="N156" s="2"/>
       <c r="O156" s="2"/>
@@ -17663,7 +17706,7 @@
         <v>76</v>
       </c>
       <c r="AF156" t="s" s="2">
-        <v>124</v>
+        <v>87</v>
       </c>
       <c r="AG156" t="s" s="2">
         <v>77</v>
@@ -17675,18 +17718,18 @@
         <v>76</v>
       </c>
       <c r="AJ156" t="s" s="2">
-        <v>125</v>
+        <v>76</v>
       </c>
       <c r="AK156" t="s" s="2">
-        <v>116</v>
+        <v>88</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B157" t="s" s="2">
-        <v>252</v>
+        <v>354</v>
       </c>
       <c r="C157" s="2"/>
       <c r="D157" t="s" s="2">
@@ -17694,10 +17737,10 @@
       </c>
       <c r="E157" s="2"/>
       <c r="F157" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G157" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="H157" t="s" s="2">
         <v>76</v>
@@ -17709,24 +17752,22 @@
         <v>76</v>
       </c>
       <c r="K157" t="s" s="2">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="L157" t="s" s="2">
-        <v>112</v>
+        <v>30</v>
       </c>
       <c r="M157" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N157" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="N157" s="2"/>
       <c r="O157" s="2"/>
       <c r="P157" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q157" s="2"/>
       <c r="R157" t="s" s="2">
-        <v>310</v>
+        <v>76</v>
       </c>
       <c r="S157" t="s" s="2">
         <v>76</v>
@@ -17756,42 +17797,42 @@
         <v>76</v>
       </c>
       <c r="AB157" t="s" s="2">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="AC157" t="s" s="2">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="AD157" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE157" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AF157" t="s" s="2">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="AG157" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AH157" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="AI157" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ157" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AK157" t="s" s="2">
-        <v>116</v>
+        <v>76</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B158" t="s" s="2">
-        <v>254</v>
+        <v>356</v>
       </c>
       <c r="C158" s="2"/>
       <c r="D158" t="s" s="2">
@@ -17799,10 +17840,10 @@
       </c>
       <c r="E158" s="2"/>
       <c r="F158" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G158" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H158" t="s" s="2">
         <v>76</v>
@@ -17814,22 +17855,24 @@
         <v>76</v>
       </c>
       <c r="K158" t="s" s="2">
-        <v>362</v>
+        <v>111</v>
       </c>
       <c r="L158" t="s" s="2">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="M158" t="s" s="2">
-        <v>121</v>
-      </c>
-      <c r="N158" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="N158" t="s" s="2">
+        <v>114</v>
+      </c>
       <c r="O158" s="2"/>
       <c r="P158" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q158" s="2"/>
       <c r="R158" t="s" s="2">
-        <v>76</v>
+        <v>361</v>
       </c>
       <c r="S158" t="s" s="2">
         <v>76</v>
@@ -17871,10 +17914,10 @@
         <v>76</v>
       </c>
       <c r="AF158" t="s" s="2">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="AG158" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="AH158" t="s" s="2">
         <v>83</v>
@@ -17883,7 +17926,7 @@
         <v>76</v>
       </c>
       <c r="AJ158" t="s" s="2">
-        <v>125</v>
+        <v>76</v>
       </c>
       <c r="AK158" t="s" s="2">
         <v>116</v>
@@ -17891,10 +17934,10 @@
     </row>
     <row r="159">
       <c r="A159" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B159" t="s" s="2">
-        <v>176</v>
+        <v>358</v>
       </c>
       <c r="C159" s="2"/>
       <c r="D159" t="s" s="2">
@@ -17902,7 +17945,7 @@
       </c>
       <c r="E159" s="2"/>
       <c r="F159" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G159" t="s" s="2">
         <v>83</v>
@@ -17917,24 +17960,22 @@
         <v>76</v>
       </c>
       <c r="K159" t="s" s="2">
-        <v>111</v>
+        <v>240</v>
       </c>
       <c r="L159" t="s" s="2">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="M159" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N159" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="N159" s="2"/>
       <c r="O159" s="2"/>
       <c r="P159" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q159" s="2"/>
       <c r="R159" t="s" s="2">
-        <v>240</v>
+        <v>76</v>
       </c>
       <c r="S159" t="s" s="2">
         <v>76</v>
@@ -17976,10 +18017,10 @@
         <v>76</v>
       </c>
       <c r="AF159" t="s" s="2">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="AG159" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AH159" t="s" s="2">
         <v>83</v>
@@ -17988,7 +18029,7 @@
         <v>76</v>
       </c>
       <c r="AJ159" t="s" s="2">
-        <v>76</v>
+        <v>125</v>
       </c>
       <c r="AK159" t="s" s="2">
         <v>116</v>
@@ -17996,12 +18037,14 @@
     </row>
     <row r="160">
       <c r="A160" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B160" t="s" s="2">
-        <v>178</v>
-      </c>
-      <c r="C160" s="2"/>
+        <v>338</v>
+      </c>
+      <c r="C160" t="s" s="2">
+        <v>368</v>
+      </c>
       <c r="D160" t="s" s="2">
         <v>76</v>
       </c>
@@ -18010,7 +18053,7 @@
         <v>77</v>
       </c>
       <c r="G160" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H160" t="s" s="2">
         <v>76</v>
@@ -18022,13 +18065,13 @@
         <v>76</v>
       </c>
       <c r="K160" t="s" s="2">
-        <v>362</v>
+        <v>90</v>
       </c>
       <c r="L160" t="s" s="2">
-        <v>120</v>
+        <v>369</v>
       </c>
       <c r="M160" t="s" s="2">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="N160" s="2"/>
       <c r="O160" s="2"/>
@@ -18079,30 +18122,30 @@
         <v>76</v>
       </c>
       <c r="AF160" t="s" s="2">
-        <v>124</v>
+        <v>95</v>
       </c>
       <c r="AG160" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH160" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="AI160" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ160" t="s" s="2">
-        <v>125</v>
+        <v>81</v>
       </c>
       <c r="AK160" t="s" s="2">
-        <v>116</v>
+        <v>76</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="s" s="2">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="B161" t="s" s="2">
-        <v>110</v>
+        <v>352</v>
       </c>
       <c r="C161" s="2"/>
       <c r="D161" t="s" s="2">
@@ -18110,7 +18153,7 @@
       </c>
       <c r="E161" s="2"/>
       <c r="F161" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G161" t="s" s="2">
         <v>83</v>
@@ -18125,24 +18168,22 @@
         <v>76</v>
       </c>
       <c r="K161" t="s" s="2">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="L161" t="s" s="2">
-        <v>112</v>
+        <v>85</v>
       </c>
       <c r="M161" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N161" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="N161" s="2"/>
       <c r="O161" s="2"/>
       <c r="P161" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q161" s="2"/>
       <c r="R161" t="s" s="2">
-        <v>164</v>
+        <v>76</v>
       </c>
       <c r="S161" t="s" s="2">
         <v>76</v>
@@ -18184,10 +18225,10 @@
         <v>76</v>
       </c>
       <c r="AF161" t="s" s="2">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="AG161" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AH161" t="s" s="2">
         <v>83</v>
@@ -18199,15 +18240,15 @@
         <v>76</v>
       </c>
       <c r="AK161" t="s" s="2">
-        <v>116</v>
+        <v>88</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="s" s="2">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="B162" t="s" s="2">
-        <v>118</v>
+        <v>354</v>
       </c>
       <c r="C162" s="2"/>
       <c r="D162" t="s" s="2">
@@ -18230,13 +18271,13 @@
         <v>76</v>
       </c>
       <c r="K162" t="s" s="2">
-        <v>362</v>
+        <v>90</v>
       </c>
       <c r="L162" t="s" s="2">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="M162" t="s" s="2">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="N162" s="2"/>
       <c r="O162" s="2"/>
@@ -18275,42 +18316,42 @@
         <v>76</v>
       </c>
       <c r="AB162" t="s" s="2">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="AC162" t="s" s="2">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="AD162" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE162" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AF162" t="s" s="2">
-        <v>124</v>
+        <v>95</v>
       </c>
       <c r="AG162" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH162" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="AI162" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ162" t="s" s="2">
-        <v>125</v>
+        <v>81</v>
       </c>
       <c r="AK162" t="s" s="2">
-        <v>116</v>
+        <v>76</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="s" s="2">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B163" t="s" s="2">
-        <v>370</v>
+        <v>356</v>
       </c>
       <c r="C163" s="2"/>
       <c r="D163" t="s" s="2">
@@ -18350,7 +18391,7 @@
       </c>
       <c r="Q163" s="2"/>
       <c r="R163" t="s" s="2">
-        <v>97</v>
+        <v>368</v>
       </c>
       <c r="S163" t="s" s="2">
         <v>76</v>
@@ -18412,10 +18453,10 @@
     </row>
     <row r="164">
       <c r="A164" t="s" s="2">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B164" t="s" s="2">
-        <v>372</v>
+        <v>358</v>
       </c>
       <c r="C164" s="2"/>
       <c r="D164" t="s" s="2">
@@ -18426,7 +18467,7 @@
         <v>77</v>
       </c>
       <c r="G164" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H164" t="s" s="2">
         <v>76</v>
@@ -18438,7 +18479,7 @@
         <v>76</v>
       </c>
       <c r="K164" t="s" s="2">
-        <v>362</v>
+        <v>119</v>
       </c>
       <c r="L164" t="s" s="2">
         <v>120</v>
@@ -18471,13 +18512,11 @@
         <v>76</v>
       </c>
       <c r="X164" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y164" t="s" s="2">
-        <v>76</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="Y164" s="2"/>
       <c r="Z164" t="s" s="2">
-        <v>76</v>
+        <v>374</v>
       </c>
       <c r="AA164" t="s" s="2">
         <v>76</v>
@@ -18515,10 +18554,10 @@
     </row>
     <row r="165">
       <c r="A165" t="s" s="2">
-        <v>115</v>
+        <v>375</v>
       </c>
       <c r="B165" t="s" s="2">
-        <v>115</v>
+        <v>340</v>
       </c>
       <c r="C165" s="2"/>
       <c r="D165" t="s" s="2">
@@ -18558,7 +18597,7 @@
       </c>
       <c r="Q165" s="2"/>
       <c r="R165" t="s" s="2">
-        <v>3</v>
+        <v>345</v>
       </c>
       <c r="S165" t="s" s="2">
         <v>76</v>
@@ -18620,10 +18659,10 @@
     </row>
     <row r="166">
       <c r="A166" t="s" s="2">
-        <v>124</v>
+        <v>376</v>
       </c>
       <c r="B166" t="s" s="2">
-        <v>124</v>
+        <v>342</v>
       </c>
       <c r="C166" s="2"/>
       <c r="D166" t="s" s="2">
@@ -18646,7 +18685,7 @@
         <v>76</v>
       </c>
       <c r="K166" t="s" s="2">
-        <v>362</v>
+        <v>377</v>
       </c>
       <c r="L166" t="s" s="2">
         <v>120</v>
@@ -18718,6 +18757,1046 @@
         <v>125</v>
       </c>
       <c r="AK166" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="s" s="2">
+        <v>378</v>
+      </c>
+      <c r="B167" t="s" s="2">
+        <v>267</v>
+      </c>
+      <c r="C167" s="2"/>
+      <c r="D167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E167" s="2"/>
+      <c r="F167" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G167" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K167" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L167" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="M167" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="N167" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="O167" s="2"/>
+      <c r="P167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q167" s="2"/>
+      <c r="R167" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="S167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF167" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG167" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH167" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ167" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK167" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="s" s="2">
+        <v>379</v>
+      </c>
+      <c r="B168" t="s" s="2">
+        <v>269</v>
+      </c>
+      <c r="C168" s="2"/>
+      <c r="D168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E168" s="2"/>
+      <c r="F168" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G168" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K168" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="L168" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="M168" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="N168" s="2"/>
+      <c r="O168" s="2"/>
+      <c r="P168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q168" s="2"/>
+      <c r="R168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF168" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="AG168" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH168" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI168" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ168" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AK168" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="s" s="2">
+        <v>380</v>
+      </c>
+      <c r="B169" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="C169" s="2"/>
+      <c r="D169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E169" s="2"/>
+      <c r="F169" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G169" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K169" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L169" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="M169" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="N169" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="O169" s="2"/>
+      <c r="P169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q169" s="2"/>
+      <c r="R169" t="s" s="2">
+        <v>256</v>
+      </c>
+      <c r="S169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF169" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG169" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH169" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ169" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK169" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="s" s="2">
+        <v>381</v>
+      </c>
+      <c r="B170" t="s" s="2">
+        <v>178</v>
+      </c>
+      <c r="C170" s="2"/>
+      <c r="D170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E170" s="2"/>
+      <c r="F170" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G170" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K170" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="L170" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="M170" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="N170" s="2"/>
+      <c r="O170" s="2"/>
+      <c r="P170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q170" s="2"/>
+      <c r="R170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF170" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="AG170" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH170" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI170" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ170" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AK170" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="s" s="2">
+        <v>382</v>
+      </c>
+      <c r="B171" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="C171" s="2"/>
+      <c r="D171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E171" s="2"/>
+      <c r="F171" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G171" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K171" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L171" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="M171" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="N171" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="O171" s="2"/>
+      <c r="P171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q171" s="2"/>
+      <c r="R171" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="S171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF171" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG171" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH171" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ171" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK171" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="s" s="2">
+        <v>383</v>
+      </c>
+      <c r="B172" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="C172" s="2"/>
+      <c r="D172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E172" s="2"/>
+      <c r="F172" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G172" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K172" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="L172" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="M172" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="N172" s="2"/>
+      <c r="O172" s="2"/>
+      <c r="P172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q172" s="2"/>
+      <c r="R172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF172" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="AG172" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH172" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI172" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ172" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AK172" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="B173" t="s" s="2">
+        <v>385</v>
+      </c>
+      <c r="C173" s="2"/>
+      <c r="D173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E173" s="2"/>
+      <c r="F173" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G173" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K173" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L173" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="M173" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="N173" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="O173" s="2"/>
+      <c r="P173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q173" s="2"/>
+      <c r="R173" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="S173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF173" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG173" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH173" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ173" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK173" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="s" s="2">
+        <v>386</v>
+      </c>
+      <c r="B174" t="s" s="2">
+        <v>387</v>
+      </c>
+      <c r="C174" s="2"/>
+      <c r="D174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E174" s="2"/>
+      <c r="F174" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G174" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K174" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="L174" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="M174" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="N174" s="2"/>
+      <c r="O174" s="2"/>
+      <c r="P174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q174" s="2"/>
+      <c r="R174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF174" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="AG174" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH174" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI174" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ174" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AK174" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="B175" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="C175" s="2"/>
+      <c r="D175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E175" s="2"/>
+      <c r="F175" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G175" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K175" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L175" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="M175" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="N175" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="O175" s="2"/>
+      <c r="P175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q175" s="2"/>
+      <c r="R175" t="s" s="2">
+        <v>3</v>
+      </c>
+      <c r="S175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF175" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG175" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH175" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ175" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK175" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="B176" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="C176" s="2"/>
+      <c r="D176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E176" s="2"/>
+      <c r="F176" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G176" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K176" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="L176" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="M176" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="N176" s="2"/>
+      <c r="O176" s="2"/>
+      <c r="P176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q176" s="2"/>
+      <c r="R176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF176" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="AG176" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH176" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI176" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ176" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AK176" t="s" s="2">
         <v>116</v>
       </c>
     </row>

</xml_diff>